<commit_message>
Day 9 learning journey - LLM Few-shot Classification vs Zero-Shot vs COT vs TOT and json format as outputsaving results to Excel file.
</commit_message>
<xml_diff>
--- a/Week2 - Prompt engineering/few_shot_complaint_classification.xlsx
+++ b/Week2 - Prompt engineering/few_shot_complaint_classification.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0.1803</v>
+        <v>0.1795</v>
       </c>
     </row>
     <row r="3">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0.1863</v>
+        <v>0.1878</v>
       </c>
     </row>
     <row r="4">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>0.1835</v>
+        <v>0.1846</v>
       </c>
     </row>
     <row r="5">
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0.1812</v>
+        <v>0.1852</v>
       </c>
     </row>
     <row r="6">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0.1852</v>
+        <v>0.1843</v>
       </c>
     </row>
   </sheetData>

</xml_diff>